<commit_message>
Consolidate KP card blocks into cards variants
Spotlight, articles, care, news, teaser (now "panels"), pillars and notices share one
content model (media cell + text cell), so they become variants of the cards block,
decorated by one shared decorator driven by a per-variant options table. Shared CSS
(list reset, stretched title link, focus ring, hairline/shadow tokens) is written once;
variant sections keep only what differs and use .cards:where(.variant) to keep their
original specificity. Default/links/bento card rules are scoped so they do not apply
to the variants.

cards-tools stays a separate block (view-all toggle + label row) and now reuses the
shared unbuttonLinks helper from scripts/shared.js. Importer parsers emit the new
variant names; health-wellness template selectors follow the rename.

The old standalone block folders are kept until the published content is updated.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-health-wellness.report.xlsx
+++ b/tools/importer/reports/import-health-wellness.report.xlsx
@@ -49,7 +49,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-10-07T21:18:53.941Z</t>
+    <t>2026-10-08T02:41:02.547Z</t>
   </si>
   <si>
     <t>Health and wellness | Kaiser Permanente</t>
@@ -70,7 +70,7 @@
     <t>northern-california</t>
   </si>
   <si>
-    <t>2026-10-07T21:18:09.417Z</t>
+    <t>2026-10-07T21:32:44.900Z</t>
   </si>
   <si>
     <t>Custom Care &amp; Coverage Just For You | Kaiser Permanente</t>

</xml_diff>